<commit_message>
Add readRawRange and extend raw_cells readCellValue fixtures.
Introduce RawVertical and readRawRange for range-based raw reads, return errors from CellRange column number helpers, and document more cell shapes (formula, error, types, whitespace) in raw_cells goldens.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/raw_cells/test_cases.xlsx
+++ b/excel/testdata/raw_cells/test_cases.xlsx
@@ -12,13 +12,20 @@
     <sheet name="vertical" sheetId="3" r:id="rId6"/>
     <sheet name="block" sheetId="4" r:id="rId7"/>
     <sheet name="two-horizontal" sheetId="5" r:id="rId8"/>
+    <sheet name="formula" sheetId="6" r:id="rId9"/>
+    <sheet name="error" sheetId="7" r:id="rId10"/>
+    <sheet name="typed-number" sheetId="8" r:id="rId11"/>
+    <sheet name="typed-date" sheetId="9" r:id="rId12"/>
+    <sheet name="text-number" sheetId="10" r:id="rId13"/>
+    <sheet name="line-break" sheetId="11" r:id="rId14"/>
+    <sheet name="whitespace" sheetId="12" r:id="rId15"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>only</t>
   </si>
@@ -36,12 +43,27 @@
   </si>
   <si>
     <t>right</t>
+  </si>
+  <si>
+    <t>00123</t>
+  </si>
+  <si>
+    <t>line
+one
+two</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  padded  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="@"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -70,8 +92,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -351,6 +379,45 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
@@ -417,4 +484,56 @@
     <mergeCell ref="D1:E1"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <f>1+2</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <f>1/0</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <v>1234.5</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1">
+        <v>45366</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>